<commit_message>
initial eda on competitor data
</commit_message>
<xml_diff>
--- a/data/Data_Dictionary.xlsx
+++ b/data/Data_Dictionary.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Hackathon\Databricks MLOps Hackathon 2025\databricks-mlops-hackathon\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ltimindtree-my.sharepoint.com/personal/ruchita_10677003_ltimindtree_com/Documents/hackthons/databricks-mlops-hackathon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79693170-4AC2-459E-9590-814B5F9959A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{79693170-4AC2-459E-9590-814B5F9959A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{528D3B1A-C2AD-4A17-AC6D-74118CC92B77}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1CF32C48-9D11-4084-B00B-D5073DE040B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{1CF32C48-9D11-4084-B00B-D5073DE040B8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Competitor_Pricing" sheetId="1" r:id="rId1"/>
-    <sheet name="Inventory" sheetId="4" r:id="rId2"/>
+    <sheet name="Inventory" sheetId="4" r:id="rId1"/>
+    <sheet name="Competitor_Pricing" sheetId="1" r:id="rId2"/>
     <sheet name="Customer_behaviour" sheetId="2" r:id="rId3"/>
     <sheet name="Sales" sheetId="3" r:id="rId4"/>
   </sheets>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="74">
   <si>
     <t>The final price of the product after applying discounts</t>
   </si>
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t>The date of the transaction</t>
+  </si>
+  <si>
+    <t>Total Records</t>
   </si>
 </sst>
 </file>
@@ -629,11 +632,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{622FD9CC-5E1D-4F6E-89B6-ABB71FCCA77D}">
-  <dimension ref="A1:D7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C72A3538-67B0-4F5F-AAE8-3B4832C46B25}">
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="49.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="100.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -658,6 +664,226 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1">
+        <v>44197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13">
+        <v>7.18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16">
+        <v>21900</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{622FD9CC-5E1D-4F6E-89B6-ABB71FCCA77D}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>70</v>
       </c>
       <c r="D2" s="1">
@@ -732,6 +958,14 @@
       </c>
       <c r="D7">
         <v>84.67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9">
+        <v>2190</v>
       </c>
     </row>
   </sheetData>
@@ -740,215 +974,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C72A3538-67B0-4F5F-AAE8-3B4832C46B25}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="1">
-        <v>44197</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>65</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>66</v>
-      </c>
-      <c r="B13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D13">
-        <v>7.18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>69</v>
-      </c>
-      <c r="D14">
-        <v>92</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8014F2D-3FF3-469D-AF82-F1C88C5995FC}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" bestFit="1" customWidth="1"/>
@@ -1082,6 +1110,14 @@
         <v>83.59</v>
       </c>
     </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11">
+        <v>365</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1089,7 +1125,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABA94502-0B82-4E9A-9FEF-C2E9570FAB2F}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -1182,6 +1218,14 @@
         <v>12</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9">
+        <v>1095</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
started eda for the sales data of tide
</commit_message>
<xml_diff>
--- a/data/Data_Dictionary.xlsx
+++ b/data/Data_Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Hackathon\Databricks MLOps Hackathon 2025\databricks-mlops-hackathon\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ltimindtree-my.sharepoint.com/personal/ruchita_10677003_ltimindtree_com/Documents/hackthons/databricks-mlops-hackathon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AAF09C-E1DD-43F0-B62D-EDC8B35AE01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{C8AAF09C-E1DD-43F0-B62D-EDC8B35AE01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DF9CC49-1BCC-4CCC-B99B-3CA210CB1D0C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{1CF32C48-9D11-4084-B00B-D5073DE040B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{1CF32C48-9D11-4084-B00B-D5073DE040B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Competitor_Pricing" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
   <si>
     <t>The final price of the product after applying discounts</t>
   </si>
@@ -258,6 +258,9 @@
   </si>
   <si>
     <t>The date of the transaction</t>
+  </si>
+  <si>
+    <t>This is the BasePrice of the product</t>
   </si>
 </sst>
 </file>
@@ -273,12 +276,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -293,9 +302,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1098,16 +1108,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABA94502-0B82-4E9A-9FEF-C2E9570FAB2F}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="57" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1121,7 +1132,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -1135,7 +1146,7 @@
         <v>44197</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1149,7 +1160,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1162,8 +1173,11 @@
       <c r="D4">
         <v>97.95</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1177,7 +1191,7 @@
         <v>97.95</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
started with basic eda on customer behaviour analysis
</commit_message>
<xml_diff>
--- a/data/Data_Dictionary.xlsx
+++ b/data/Data_Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ltimindtree-my.sharepoint.com/personal/ruchita_10677003_ltimindtree_com/Documents/hackthons/databricks-mlops-hackathon/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{C8AAF09C-E1DD-43F0-B62D-EDC8B35AE01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DF9CC49-1BCC-4CCC-B99B-3CA210CB1D0C}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{C8AAF09C-E1DD-43F0-B62D-EDC8B35AE01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB15DDDA-E2C6-40AF-A1B7-95DF5EC56AAA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{1CF32C48-9D11-4084-B00B-D5073DE040B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{1CF32C48-9D11-4084-B00B-D5073DE040B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Competitor_Pricing" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="76">
   <si>
     <t>The final price of the product after applying discounts</t>
   </si>
@@ -261,6 +261,12 @@
   </si>
   <si>
     <t>This is the BasePrice of the product</t>
+  </si>
+  <si>
+    <t>how many times an ad was clicked to the viewed</t>
+  </si>
+  <si>
+    <t>Future advertisecontent duration</t>
   </si>
 </sst>
 </file>
@@ -967,15 +973,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8014F2D-3FF3-469D-AF82-F1C88C5995FC}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="67.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="73.28515625" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="54" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -989,7 +996,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1003,7 +1010,7 @@
         <v>44197</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1016,8 +1023,11 @@
       <c r="D3">
         <v>3.5999999999999997E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1031,7 +1041,7 @@
         <v>0.61299999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1045,7 +1055,7 @@
         <v>0.49680000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1059,7 +1069,7 @@
         <v>0.38540000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -1073,7 +1083,7 @@
         <v>0.51980000000000004</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1087,7 +1097,7 @@
         <v>0.24110000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1099,6 +1109,9 @@
       </c>
       <c r="D9">
         <v>83.59</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1113,7 +1126,7 @@
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.5703125" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35.42578125" customWidth="1"/>
   </cols>

</xml_diff>